<commit_message>
Add Lesson 4, 5
</commit_message>
<xml_diff>
--- a/data/2026_F_M_Words.xlsx
+++ b/data/2026_F_M_Words.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\word-tester\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C88E6E4-A4B7-4550-A1D0-BF1F20DFEC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C6F455-3DEB-47DA-8A83-D44F67733A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A78F504C-B3D1-44D7-A0F0-C4A481C15F08}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A78F504C-B3D1-44D7-A0F0-C4A481C15F08}"/>
   </bookViews>
   <sheets>
     <sheet name="Chapter 1" sheetId="1" r:id="rId1"/>
     <sheet name="Chapter 2" sheetId="2" r:id="rId2"/>
     <sheet name="Chatper 3" sheetId="3" r:id="rId3"/>
+    <sheet name="Chapter 4" sheetId="4" r:id="rId4"/>
+    <sheet name="Chapter 5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="533">
   <si>
     <t>단어 (Word)</t>
   </si>
@@ -966,13 +969,1024 @@
   <si>
     <t>check out</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>• Shawn attained his goal of getting straight A's.</t>
+  </si>
+  <si>
+    <t>• The wild deer managed to elude the hunters.</t>
+  </si>
+  <si>
+    <t>• A helicopter can hover above a building.</t>
+  </si>
+  <si>
+    <t>• You can use a bicycle pump to inflate the flat tire with air.</t>
+  </si>
+  <si>
+    <t>jeopardy [n.]</t>
+  </si>
+  <si>
+    <t>Danger</t>
+  </si>
+  <si>
+    <t>• Pollution and severe weather put the sea turtles in jeopardy.</t>
+  </si>
+  <si>
+    <t>• The rock slide threatened to put their lives in jeopardy.</t>
+  </si>
+  <si>
+    <t>To put in danger</t>
+  </si>
+  <si>
+    <t>• Bad weather could jeopardize the outdoor wedding plans.</t>
+  </si>
+  <si>
+    <t>moor [v.]</t>
+  </si>
+  <si>
+    <t>To hold in place with ropes or anchors</t>
+  </si>
+  <si>
+    <t>• The captain used strong ropes to moor the boat to the dock before the storm.</t>
+  </si>
+  <si>
+    <t>A place to which a boat or aircraft can be moored</t>
+  </si>
+  <si>
+    <t>• A mooring holds the boat safely in the harbor.</t>
+  </si>
+  <si>
+    <t>plummet [v.]</t>
+  </si>
+  <si>
+    <t>To fall suddenly towards the earth</t>
+  </si>
+  <si>
+    <t>• If you drop a heavy anchor into the ocean, it will plummet to the seabed.</t>
+  </si>
+  <si>
+    <t>• The temperature began to plummet at sunset.</t>
+  </si>
+  <si>
+    <t>pollute [v.]</t>
+  </si>
+  <si>
+    <t>To make dirty or impure</t>
+  </si>
+  <si>
+    <t>• Careless dumping of industrial waste will pollute the local groundwater.</t>
+  </si>
+  <si>
+    <t>• Toxic chemicals can pollute the fresh stream.</t>
+  </si>
+  <si>
+    <t>The action of polluting; the state of being polluted</t>
+  </si>
+  <si>
+    <t>• Air pollution is a major problem in many big cities.</t>
+  </si>
+  <si>
+    <t>propel [v.]</t>
+  </si>
+  <si>
+    <t>To push or drive forward</t>
+  </si>
+  <si>
+    <t>• Two giant engines work together to propel the airplane forward.</t>
+  </si>
+  <si>
+    <t>• Two powerful engines propel the speedboat.</t>
+  </si>
+  <si>
+    <t>stationary [adj.]</t>
+  </si>
+  <si>
+    <t>1) Not moving. 2) Not changing.</t>
+  </si>
+  <si>
+    <t>• The target remained stationary during practice.</t>
+  </si>
+  <si>
+    <t>• The bus remained stationary at the red light until it turned green.</t>
+  </si>
+  <si>
+    <t>Of the highest quality; grand; splendid</t>
+  </si>
+  <si>
+    <t>• The orchestra gave a superb performance that earned a standing ovation.</t>
+  </si>
+  <si>
+    <t>• The view from the mountaintop was superb.</t>
+  </si>
+  <si>
+    <t>come out</t>
+  </si>
+  <si>
+    <t>attain [v.]</t>
+  </si>
+  <si>
+    <t>buffet [n.]</t>
+  </si>
+  <si>
+    <t>buffet [v.]</t>
+  </si>
+  <si>
+    <t>elusive [adj.]</t>
+  </si>
+  <si>
+    <t>jeopardize [v.]</t>
+  </si>
+  <si>
+    <t>mooring [n.]</t>
+  </si>
+  <si>
+    <t>pollution [n.]</t>
+  </si>
+  <si>
+    <t>swivel [n.]</t>
+  </si>
+  <si>
+    <t>swivel [v.]</t>
+  </si>
+  <si>
+    <t>• The hot air balloon floated aloft above the fields, offering a beautiful view.</t>
+  </si>
+  <si>
+    <t>• The eagle soared aloft, gliding through the sky with its wings spread wide.</t>
+  </si>
+  <si>
+    <t>• The paper airplane was thrown aloft, circling around before landing.</t>
+  </si>
+  <si>
+    <t>aloft [adv.]</t>
+  </si>
+  <si>
+    <t>Up in the air, especially in flight</t>
+  </si>
+  <si>
+    <t>• A strong breeze kept the kites aloft.</t>
+  </si>
+  <si>
+    <t>1) To reach; to arrive at</t>
+  </si>
+  <si>
+    <t>• Redwood trees attain heights of over three hundred feet.</t>
+  </si>
+  <si>
+    <t>2) To achieve</t>
+  </si>
+  <si>
+    <t>1) A piece of furniture with drawers and shelves for storage and display</t>
+  </si>
+  <si>
+    <t>• This splendid antique buffet contains a valuable collection of china.</t>
+  </si>
+  <si>
+    <t>2) A meal laid out for guests to help themselves</t>
+  </si>
+  <si>
+    <t>• The abundance of food at the buffet allowed people to go back for second or third helpings.</t>
+  </si>
+  <si>
+    <t>3) To pound repeatedly; to batter</t>
+  </si>
+  <si>
+    <t>• High winds and waves buffeted the ship during the storm.</t>
+  </si>
+  <si>
+    <t>elude [v.]</t>
+  </si>
+  <si>
+    <t>To escape by being quick or clever</t>
+  </si>
+  <si>
+    <t>• The mouse eluded the cat by slipping through a crack in the wall.</t>
+  </si>
+  <si>
+    <t>1) Hard to find or capture</t>
+  </si>
+  <si>
+    <t>• The elusive outlaws were familiar with the terrain while those pursuing them were not.</t>
+  </si>
+  <si>
+    <t>2) Hard to explain, make clear, or understand</t>
+  </si>
+  <si>
+    <t>• Albert Einstein's connection between energy and the speed of light is too elusive for most nonscientists to grasp.</t>
+  </si>
+  <si>
+    <t>flammable [adj.]</t>
+  </si>
+  <si>
+    <t>Able to catch fire easily</t>
+  </si>
+  <si>
+    <t>• Children's night clothes must be fireproofed so they are not flammable.</t>
+  </si>
+  <si>
+    <t>hover [v.]</t>
+  </si>
+  <si>
+    <t>To remain in place over an object or location</t>
+  </si>
+  <si>
+    <t>• Hummingbirds hover by beating their wings sixty times a second.</t>
+  </si>
+  <si>
+    <t>inflate [v.]</t>
+  </si>
+  <si>
+    <t>To fill with air or other gas</t>
+  </si>
+  <si>
+    <t>• Inflate the tires to the correct pressure.</t>
+  </si>
+  <si>
+    <t>**antic [n.]</t>
+  </si>
+  <si>
+    <t>(usually plural)</t>
+  </si>
+  <si>
+    <r>
+      <t>A playful or funny act</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[1]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The antics of the clown made the crowd roar with laughter[1].</t>
+  </si>
+  <si>
+    <t>• The puppy’s playful antic of chasing its tail entertained the whole family[1].</t>
+  </si>
+  <si>
+    <t>**attire [n.]</t>
+  </si>
+  <si>
+    <r>
+      <t>Clothes, especially fine and expensive clothes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[2]</t>
+    </r>
+  </si>
+  <si>
+    <t>• One often needs special attire to be in a wedding party[2].</t>
+  </si>
+  <si>
+    <t>**attire [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>To dress up or be dressed up</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[2]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The designer attired the models in shirts and trousers for the fashion show[2].</t>
+  </si>
+  <si>
+    <t>captivate [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>To please greatly; to win over by special charm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[3]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The cast’s superb acting captivated the audience[3].</t>
+  </si>
+  <si>
+    <t>• The storyteller’s voice was so powerful that it could captivate an entire room[3].</t>
+  </si>
+  <si>
+    <t>• Her singing was so beautiful that it would captivate anyone listening[3].</t>
+  </si>
+  <si>
+    <t>deft [adj.]</t>
+  </si>
+  <si>
+    <r>
+      <t>Quick and sure; skillful at handling</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[3]</t>
+    </r>
+  </si>
+  <si>
+    <t>• A deft juggler can keep five or more objects in the air at one time[3].</t>
+  </si>
+  <si>
+    <t>• The chef’s deft hands quickly chopped the vegetables into perfect slices[3].</t>
+  </si>
+  <si>
+    <t>• He showed deft skill when playing the guitar, impressing everyone[3].</t>
+  </si>
+  <si>
+    <t>• The surgeon's deft fingers worked carefully during the operation[4].</t>
+  </si>
+  <si>
+    <t>diligent [adj.]</t>
+  </si>
+  <si>
+    <r>
+      <t>Working with great care and effort</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[5]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Diligent students succeed in reaching their goals[5]. / Diligent students usually attain high marks[6].</t>
+  </si>
+  <si>
+    <t>• The gardener was diligent in taking care of the plants, watering them every day[5].</t>
+  </si>
+  <si>
+    <t>• The diligent nurse carefully checked on each patient throughout her shift[5].</t>
+  </si>
+  <si>
+    <t>**eclipse [n.]</t>
+  </si>
+  <si>
+    <r>
+      <t>The total or partial hiding of one heavenly body by another</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[5]</t>
+    </r>
+  </si>
+  <si>
+    <t>• An eclipse of the sun occurs when the moon passes directly in front of it[5].</t>
+  </si>
+  <si>
+    <t>**eclipse [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>To do or be better than; to outshine</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[6][7]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Her latest novel eclipses all her previous work[6][7].</t>
+  </si>
+  <si>
+    <t>evolve [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>To develop and change gradually over time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[6][8]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Some scientists think that modern birds may have evolved from dinosaurs[6][8].</t>
+  </si>
+  <si>
+    <t>**evolution [n.]</t>
+  </si>
+  <si>
+    <t>(evolve의 변화형)</t>
+  </si>
+  <si>
+    <r>
+      <t>The changes that take place as something evolves</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[6][8]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The evolution of aircraft from the Wright brothers' flimsy plane to the modern jet airplane occurred over an incredibly short time[8][9].</t>
+  </si>
+  <si>
+    <t>innate [adj.]</t>
+  </si>
+  <si>
+    <r>
+      <t>Having from birth; occurring naturally rather than being learned</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[8][9]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Mozart’s innate musical ability showed itself at a very early age[8][9].</t>
+  </si>
+  <si>
+    <t>inscribe [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>To write, print, or etch into as a permanent record</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[8][10]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Most of the gravestones were inscribed with the person’s name[8][10].</t>
+  </si>
+  <si>
+    <t>• We decided to inscribe our names on the tree to remember our friendship[10].</t>
+  </si>
+  <si>
+    <t>• The ring had their wedding date inscribed on the inside[10].</t>
+  </si>
+  <si>
+    <t>**inscription [n.]</t>
+  </si>
+  <si>
+    <t>(inscribe의 변화형)</t>
+  </si>
+  <si>
+    <r>
+      <t>The act of inscribing or what is inscribed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[10][11]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Coins of the United States bear the inscription "E Pluribus Unum."[10][11]</t>
+  </si>
+  <si>
+    <t>• The golden pocket watch had a beautiful inscription on its back[10].</t>
+  </si>
+  <si>
+    <t>**posture [n.]</t>
+  </si>
+  <si>
+    <r>
+      <t>The way one holds one’s body; a pose or position</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[12]</t>
+    </r>
+  </si>
+  <si>
+    <t>• You can improve your posture by throwing your shoulders back[12].</t>
+  </si>
+  <si>
+    <t>• The soldier stood with perfect posture during the ceremony[12].</t>
+  </si>
+  <si>
+    <t>**posture [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>To assume a particular position, especially a pretended one</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[12]</t>
+    </r>
+  </si>
+  <si>
+    <t>• They postured as my friends while secretly talking behind my back[12].</t>
+  </si>
+  <si>
+    <t>**shroud [n.]</t>
+  </si>
+  <si>
+    <r>
+      <t>1) Something that covers or hides from view</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][13]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2) Cloth used to wrap a dead body before burial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][13]</t>
+    </r>
+  </si>
+  <si>
+    <t>• A shroud of mystery surrounds the couple’s appearance[13].</t>
+  </si>
+  <si>
+    <t>• The ghost story described how the spirit was wrapped in a shroud[13].</t>
+  </si>
+  <si>
+    <t>**shroud [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>To block from sight</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][13]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Dense fog on the river shrouded the tugboats[11][13].</t>
+  </si>
+  <si>
+    <t>stifle [v.]</t>
+  </si>
+  <si>
+    <r>
+      <t>1) To cut off the air from; to smother</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][14]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2) To hold back; to check</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][14]</t>
+    </r>
+  </si>
+  <si>
+    <t>• Thick smoke stifled those who sat around the campfire / remained in the burning building[11][14].</t>
+  </si>
+  <si>
+    <t>• The spectators tried to stifle their yawns during the lengthy ceremony[11][14].</t>
+  </si>
+  <si>
+    <t>• She tried to stifle a laugh during the serious movie, but it was too funny[14].</t>
+  </si>
+  <si>
+    <t>• She covered her mouth to stifle the sneeze during the quiet concert[14].</t>
+  </si>
+  <si>
+    <t>tentative [adj.]</t>
+  </si>
+  <si>
+    <r>
+      <t>Not fully worked out or final; hesitating or uncertain</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][14]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The deadline is tentative and may be extended[11][14].</t>
+  </si>
+  <si>
+    <t>• We made a tentative plan to meet at the park, but it might change if it rains[14].</t>
+  </si>
+  <si>
+    <t>• Her tentative steps on the ice showed she was nervous about slipping[15].</t>
+  </si>
+  <si>
+    <t>• He offered a tentative smile when he met the new students in class[15].</t>
+  </si>
+  <si>
+    <t>tranquil [adj.]</t>
+  </si>
+  <si>
+    <r>
+      <t>Calm; peaceful</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][15]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The sea was tranquil with no hint of the approaching storm[11][15].</t>
+  </si>
+  <si>
+    <t>• She felt tranquil as she listened to the soft sounds of nature in the forest[15].</t>
+  </si>
+  <si>
+    <t>• Listening to tranquil music helped her focus while studying[15].</t>
+  </si>
+  <si>
+    <t>**tranquility [n.]</t>
+  </si>
+  <si>
+    <r>
+      <t>The state of being tranquil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][15]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The simple act of sipping tea by the fireplace brought a feeling of tranquility to his evenings[15].</t>
+  </si>
+  <si>
+    <t>versatile [adj.]</t>
+  </si>
+  <si>
+    <r>
+      <t>Able to do many different things or to be used in many different ways</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][16]</t>
+    </r>
+  </si>
+  <si>
+    <t>• She is a versatile musician who can play eight instruments[11][16].</t>
+  </si>
+  <si>
+    <t>**versatility [n.]</t>
+  </si>
+  <si>
+    <r>
+      <t>The state or condition of being versatile</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[11][16]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The tomato’s versatility and distinct flavor make it a favorite of many cooks[11][16].</t>
+  </si>
+  <si>
+    <r>
+      <t>1) To emerge or appear, often from a hidden or concealed place.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[17]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The sun came out from behind the clouds, brightening the day[17].</t>
+  </si>
+  <si>
+    <r>
+      <t>2) To be released or published, such as in the case of information, news, or a product becoming available to the public.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[17]</t>
+    </r>
+  </si>
+  <si>
+    <t>• The new book by the famous author will come out next month[17].</t>
+  </si>
+  <si>
+    <t>1) To emerge or appear, often from a hidden or concealed place.</t>
+  </si>
+  <si>
+    <t>• The sun came out from behind the clouds, brightening the day.</t>
+  </si>
+  <si>
+    <t>2) To be released or published, such as in the case of information, news, or a product becoming available to the public.</t>
+  </si>
+  <si>
+    <t>• The new book by the famous author will come out next month.</t>
+  </si>
+  <si>
+    <t>come over</t>
+  </si>
+  <si>
+    <t>1) To visit someone's home or location, often informally or without prior arrangement.</t>
+  </si>
+  <si>
+    <t>• I'd love for you to come over for dinner tonight; I'll cook your favorite meal.</t>
+  </si>
+  <si>
+    <t>2) To be influenced by a particular feeling or emotion, especially suddenly or unexpectedly.</t>
+  </si>
+  <si>
+    <t>• When she heard the news, a sense of sadness came over her.</t>
+  </si>
+  <si>
+    <t>come round</t>
+  </si>
+  <si>
+    <t>1) To visit someone's home or a place for a social visit, often when it's not planned or expected.</t>
+  </si>
+  <si>
+    <t>• We were just sitting down to dinner when our friends decided to come round for a surprise visit.</t>
+  </si>
+  <si>
+    <t>2) To regain consciousness after fainting or being unconscious.</t>
+  </si>
+  <si>
+    <t>• After he fainted at the sight of blood, it took a few minutes for him to come round.</t>
+  </si>
+  <si>
+    <t>dress up</t>
+  </si>
+  <si>
+    <t>1) To wear formal or fancy clothing, often in a special or elegant manner, especially for a special occasion or event.</t>
+  </si>
+  <si>
+    <t>• I like to dress up in a fancy dress and go out for a nice dinner on my birthday.</t>
+  </si>
+  <si>
+    <t>2) To put on a costume or disguise, often for fun or as part of a themed event.</t>
+  </si>
+  <si>
+    <t>• The children love to dress up in costumes for Halloween.</t>
+  </si>
+  <si>
+    <t>fall out</t>
+  </si>
+  <si>
+    <t>1) To drop or come loose from a place or position, often unintentionally.</t>
+  </si>
+  <si>
+    <t>• The book fell out of the crowded bookshelf when he tried to retrieve it.</t>
+  </si>
+  <si>
+    <t>2) To have a disagreement or argument with someone, resulting in a strained or broken relationship.</t>
+  </si>
+  <si>
+    <t>• Jane and Sarah used to be best friends, but they fell out over a misunderstanding and haven't spoken in months.</t>
+  </si>
+  <si>
+    <t>1) To become happier or feel better, especially after feeling sad or upset.</t>
+  </si>
+  <si>
+    <t>• Tim was feeling down after losing the game, but his friends helped him cheer up by telling jokes.</t>
+  </si>
+  <si>
+    <t>2) To make someone else feel happier or better when they are upset or sad.</t>
+  </si>
+  <si>
+    <t>• To cheer up his little brother, Tim gave him his favorite toy to play with.</t>
+  </si>
+  <si>
+    <t>1) To make a place tidy by removing dirt, mess, or clutter.</t>
+  </si>
+  <si>
+    <t>• After the party, we all helped clean up the living room to make it tidy again.</t>
+  </si>
+  <si>
+    <t>2) To wash oneself or get rid of dirt, especially after getting dirty.</t>
+  </si>
+  <si>
+    <t>• After playing in the mud, Tim had to clean up before coming inside the house.</t>
+  </si>
+  <si>
+    <t>3) To finish something thoroughly or completely, often related to success or winning.</t>
+  </si>
+  <si>
+    <t>• The team cleaned up at the school’s science fair, winning first place in every category.</t>
+  </si>
+  <si>
+    <t>1) To return to a place after being away.</t>
+  </si>
+  <si>
+    <t>• Sarah left her book at the park, so she had to come back to get it.</t>
+  </si>
+  <si>
+    <t>2) To regain strength, popularity, or success after a decline or loss.</t>
+  </si>
+  <si>
+    <t>• After losing the first half of the game, the team made an amazing effort to come back and win.</t>
+  </si>
+  <si>
+    <t>3) To remember or think of something again after a period of forgetting.</t>
+  </si>
+  <si>
+    <t>• The details of the story started to come back to Tim as he reread the book.</t>
+  </si>
+  <si>
+    <t>1) To move from a higher place to a lower place.</t>
+  </si>
+  <si>
+    <t>• Tim climbed the tree but had to come down when it started raining.</t>
+  </si>
+  <si>
+    <t>2) To decrease in amount, price, or level.</t>
+  </si>
+  <si>
+    <t>• The temperature will come down later today, making it cooler for the picnic.</t>
+  </si>
+  <si>
+    <t>3) To pass through generations or from a past time to the present.</t>
+  </si>
+  <si>
+    <t>• This family recipe has come down from my grandmother, and now we use it for every holiday.</t>
+  </si>
+  <si>
+    <t>1) To enter a place, such as a room or building.</t>
+  </si>
+  <si>
+    <t>• When you arrive, please knock and then come in quietly.</t>
+  </si>
+  <si>
+    <t>2) To be received or to arrive, often used for things like messages or results.</t>
+  </si>
+  <si>
+    <t>• The test results will come in tomorrow, and we’ll know how everyone did.</t>
+  </si>
+  <si>
+    <t>3) To be useful or play an important role.</t>
+  </si>
+  <si>
+    <t>• The flashlight will come in handy during the camping trip when it gets dark.</t>
+  </si>
+  <si>
+    <t>superb [adj.]</t>
+  </si>
+  <si>
+    <t>1) A fastening that allows any part joined to it to swing freely</t>
+  </si>
+  <si>
+    <t>• This chair has a swivel that enables it to turn in a full circle.</t>
+  </si>
+  <si>
+    <t>2) To turn freely around a fixed point</t>
+  </si>
+  <si>
+    <t>• Owls can swivel their heads to look behind them.</t>
+  </si>
+  <si>
+    <t>come back</t>
+  </si>
+  <si>
+    <t>clean up</t>
+  </si>
+  <si>
+    <t>cheer up</t>
+  </si>
+  <si>
+    <t>come down</t>
+  </si>
+  <si>
+    <t>come in</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1005,21 +2019,108 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F9FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDADCE0"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDADCE0"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFDADCE0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFDADCE0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDADCE0"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDADCE0"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFDADCE0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDADCE0"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDADCE0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDADCE0"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDADCE0"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFDADCE0"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1028,7 +2129,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1046,6 +2147,57 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2644,4 +3796,1155 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9188F4A8-63B1-411E-8048-C7C5332A34AE}">
+  <dimension ref="A1:C52"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.25" style="16" customWidth="1"/>
+    <col min="2" max="2" width="60.875" customWidth="1"/>
+    <col min="3" max="3" width="88.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="9" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="9" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="10" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="18" t="s">
+        <v>366</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="19"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="19"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="19"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="10" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="10" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="19"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="10" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="19"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="10" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="19"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="10" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="18" t="s">
+        <v>523</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="19"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="10" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>526</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>497</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>501</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>509</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>513</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>517</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52"/>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:B35"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" copies="5" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3C92B98-7932-44B2-B410-366A0BA544E3}">
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.375" customWidth="1"/>
+    <col min="2" max="2" width="81.125" customWidth="1"/>
+    <col min="3" max="3" width="113.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>374</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="9" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>377</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="18" t="s">
+        <v>383</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="9" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="19"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="10" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="9" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="9" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="10" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>395</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="9" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="10" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="12" t="s">
+        <v>405</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>410</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="22"/>
+    </row>
+    <row r="21" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="12" t="s">
+        <v>412</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>413</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="18" t="s">
+        <v>415</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="9" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="10" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>422</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="B26" s="19"/>
+      <c r="C26" s="10" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>426</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="11"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="10" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>434</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="18" t="s">
+        <v>440</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="20"/>
+      <c r="B34" s="14" t="s">
+        <v>442</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="20"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="9" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="19"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="10" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="18" t="s">
+        <v>447</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>448</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="20"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="9" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="20"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="9" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="19"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="10" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>454</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="20"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="9" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="19"/>
+      <c r="B43" s="19"/>
+      <c r="C43" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="8" t="s">
+        <v>458</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="12" t="s">
+        <v>461</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>462</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="8" t="s">
+        <v>464</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="7" t="s">
+        <v>475</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="7" t="s">
+        <v>475</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="30" x14ac:dyDescent="0.3">
+      <c r="A58" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>494</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="A37:A40"/>
+    <mergeCell ref="B37:B40"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>